<commit_message>
updated some raw data
</commit_message>
<xml_diff>
--- a/raw/Wetland_vege_summs_newboundary.xlsx
+++ b/raw/Wetland_vege_summs_newboundary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24527"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unsw-my.sharepoint.com/personal/z5204897_ad_unsw_edu_au1/Documents/Desktop/Honours_UNSW/Assessment/cumbung_assessment/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="280" documentId="8_{3811E941-8018-40D3-99B0-7EE44C8386A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D57FC45D-7C30-492D-BE87-C9A475B53110}"/>
+  <xr:revisionPtr revIDLastSave="289" documentId="8_{3811E941-8018-40D3-99B0-7EE44C8386A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B93B3249-B925-4E4E-B641-BC76D0F5B1A7}"/>
   <bookViews>
-    <workbookView xWindow="10968" yWindow="132" windowWidth="12048" windowHeight="11556" activeTab="2" xr2:uid="{2C41654C-0AB6-4DBC-8362-6A247B7F29DA}"/>
+    <workbookView xWindow="360" yWindow="372" windowWidth="20352" windowHeight="13164" activeTab="2" xr2:uid="{2C41654C-0AB6-4DBC-8362-6A247B7F29DA}"/>
   </bookViews>
   <sheets>
     <sheet name="All_ANAE" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1115" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1115" uniqueCount="89">
   <si>
     <t>ANAE_TYPE</t>
   </si>
@@ -303,6 +303,9 @@
   </si>
   <si>
     <t>Macquarie marshes- changed permanent wetlands into permanent tall emergent marshes</t>
+  </si>
+  <si>
+    <t>Other wetland types</t>
   </si>
 </sst>
 </file>
@@ -4049,7 +4052,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>39</v>
@@ -4109,7 +4112,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>32</v>
@@ -4184,7 +4187,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>44</v>
@@ -4259,7 +4262,7 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>10</v>
@@ -4332,7 +4335,7 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>35</v>
@@ -4430,7 +4433,7 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>40</v>
@@ -4528,7 +4531,7 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="B38" s="6" t="s">
         <v>51</v>
@@ -4584,7 +4587,7 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>43</v>
@@ -4612,7 +4615,7 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="B44" s="4" t="s">
         <v>3</v>

</xml_diff>